<commit_message>
Fusion modifications PC local + corrections titre/source + nouvelles vues + fichier migration
</commit_message>
<xml_diff>
--- a/Donnees/Statisiques Environnementales et de la  gouvernace/Gouvernance/IND-Gouvernace 14-08-2025xlsb.xlsx
+++ b/Donnees/Statisiques Environnementales et de la  gouvernace/Gouvernance/IND-Gouvernace 14-08-2025xlsb.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansad\OneDrive\Desktop\Gouvernance\Mon Travail\Annuaires et tableaux de service\Telech site\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\Ansade_Project\Donnees\Statisiques Environnementales et de la  gouvernace\Gouvernance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C29DEA1-5AF3-4A9F-8172-E05F617EC597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729039A5-D801-4983-8696-297C90A7B17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TSN1" sheetId="4" r:id="rId1"/>
@@ -39,23 +39,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="176">
   <si>
     <t>Source: https://data.unhcr.org/fr/country/mrt</t>
   </si>
@@ -236,9 +225,6 @@
   </si>
   <si>
     <t>Sièges</t>
-  </si>
-  <si>
-    <t>Source: Source: CENI et old.ami.mr</t>
   </si>
   <si>
     <t>Taux de participation</t>
@@ -1892,14 +1878,14 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27.65" customHeight="1" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="27.6" customHeight="1" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" thickBot="1" x14ac:dyDescent="1">
+    <row r="1" spans="1:8" ht="30.6" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A1" s="154" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B1" s="154"/>
       <c r="C1" s="154"/>
@@ -1909,7 +1895,7 @@
       <c r="G1" s="154"/>
       <c r="H1" s="8"/>
     </row>
-    <row r="2" spans="1:8" ht="27.65" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
@@ -1932,7 +1918,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="27.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="3" spans="1:8" ht="27.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -1955,7 +1941,7 @@
         <v>116055</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="27.65" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1976,18 +1962,18 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:T8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
     <col min="1" max="1" width="20" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="18" width="11.08984375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="19.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="11.54296875" style="1"/>
+    <col min="2" max="2" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="18" width="11.109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:20" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="33" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
@@ -2008,66 +1994,66 @@
       <c r="R1" s="8"/>
       <c r="S1" s="8"/>
     </row>
-    <row r="2" spans="1:20" ht="81" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:20" ht="79.2" x14ac:dyDescent="0.7">
       <c r="A2" s="140" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="110" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="111" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="111" t="s">
+      <c r="D2" s="110" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="110" t="s">
-        <v>84</v>
-      </c>
-      <c r="E2" s="29" t="s">
+      <c r="F2" s="63" t="s">
         <v>105</v>
       </c>
-      <c r="F2" s="63" t="s">
+      <c r="G2" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="G2" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="H2" s="29" t="s">
+      <c r="I2" s="63" t="s">
         <v>107</v>
       </c>
-      <c r="I2" s="63" t="s">
+      <c r="J2" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="K2" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="K2" s="29" t="s">
+      <c r="L2" s="63" t="s">
         <v>109</v>
       </c>
-      <c r="L2" s="63" t="s">
+      <c r="M2" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="N2" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="M2" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="N2" s="29" t="s">
+      <c r="O2" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="O2" s="63" t="s">
+      <c r="P2" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q2" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="P2" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q2" s="29" t="s">
+      <c r="R2" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="R2" s="63" t="s">
-        <v>114</v>
-      </c>
       <c r="S2" s="29" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.9">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.7">
       <c r="A3" s="60" t="s">
         <v>34</v>
       </c>
@@ -2125,7 +2111,7 @@
         <v>1194</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.7">
       <c r="A4" s="60" t="s">
         <v>33</v>
       </c>
@@ -2183,7 +2169,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.7">
       <c r="A5" s="60" t="s">
         <v>32</v>
       </c>
@@ -2243,7 +2229,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.7">
       <c r="A6" s="60" t="s">
         <v>31</v>
       </c>
@@ -2301,7 +2287,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.7">
       <c r="A7" s="60" t="s">
         <v>30</v>
       </c>
@@ -2361,7 +2347,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="15.65" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A8" s="50" t="s">
         <v>28</v>
       </c>
@@ -2397,15 +2383,15 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:P12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="16" width="16.1796875" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="16" width="16.21875" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30" thickBot="1" x14ac:dyDescent="1">
+    <row r="1" spans="1:16" ht="30.6" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A1" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B1" s="54"/>
       <c r="C1" s="54"/>
@@ -2423,87 +2409,87 @@
       <c r="O1" s="55"/>
       <c r="P1" s="55"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.7">
       <c r="A2" s="141" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="159" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C2" s="160"/>
       <c r="D2" s="161"/>
       <c r="E2" s="159" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F2" s="160"/>
       <c r="G2" s="161"/>
       <c r="H2" s="156" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I2" s="157"/>
       <c r="J2" s="158"/>
       <c r="K2" s="156" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L2" s="157"/>
       <c r="M2" s="158"/>
       <c r="N2" s="162" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O2" s="163"/>
       <c r="P2" s="164"/>
     </row>
-    <row r="3" spans="1:16" ht="81" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:16" ht="79.2" x14ac:dyDescent="0.7">
       <c r="A3" s="142" t="s">
         <v>35</v>
       </c>
       <c r="B3" s="78" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="79" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="79" t="s">
+      <c r="D3" s="78" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="78" t="s">
+      <c r="E3" s="78" t="s">
         <v>117</v>
       </c>
-      <c r="E3" s="78" t="s">
+      <c r="F3" s="79" t="s">
         <v>118</v>
       </c>
-      <c r="F3" s="79" t="s">
+      <c r="G3" s="78" t="s">
         <v>119</v>
       </c>
-      <c r="G3" s="78" t="s">
+      <c r="H3" s="78" t="s">
         <v>120</v>
       </c>
-      <c r="H3" s="78" t="s">
+      <c r="I3" s="79" t="s">
         <v>121</v>
       </c>
-      <c r="I3" s="79" t="s">
+      <c r="J3" s="78" t="s">
         <v>122</v>
       </c>
-      <c r="J3" s="78" t="s">
+      <c r="K3" s="78" t="s">
         <v>123</v>
       </c>
-      <c r="K3" s="78" t="s">
+      <c r="L3" s="79" t="s">
         <v>124</v>
       </c>
-      <c r="L3" s="79" t="s">
+      <c r="M3" s="78" t="s">
         <v>125</v>
       </c>
-      <c r="M3" s="78" t="s">
+      <c r="N3" s="78" t="s">
         <v>126</v>
       </c>
-      <c r="N3" s="78" t="s">
+      <c r="O3" s="79" t="s">
         <v>127</v>
       </c>
-      <c r="O3" s="79" t="s">
+      <c r="P3" s="78" t="s">
         <v>128</v>
       </c>
-      <c r="P3" s="78" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.9">
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.7">
       <c r="A4" s="75" t="s">
         <v>34</v>
       </c>
@@ -2556,7 +2542,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.7">
       <c r="A5" s="75" t="s">
         <v>33</v>
       </c>
@@ -2609,7 +2595,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.7">
       <c r="A6" s="75" t="s">
         <v>32</v>
       </c>
@@ -2662,7 +2648,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.7">
       <c r="A7" s="75" t="s">
         <v>31</v>
       </c>
@@ -2715,7 +2701,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.7">
       <c r="A8" s="75" t="s">
         <v>30</v>
       </c>
@@ -2768,7 +2754,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.7">
       <c r="A9" s="75" t="s">
         <v>37</v>
       </c>
@@ -2807,7 +2793,7 @@
       <c r="O9" s="73"/>
       <c r="P9" s="73"/>
     </row>
-    <row r="10" spans="1:16" ht="27.5" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="10" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A10" s="72" t="s">
         <v>4</v>
       </c>
@@ -2857,7 +2843,7 @@
         <v>15.203531142717001</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="11" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A11" s="67" t="s">
         <v>28</v>
       </c>
@@ -2877,7 +2863,7 @@
       <c r="O11" s="155"/>
       <c r="P11" s="155"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.9">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.7">
       <c r="O12" s="109"/>
     </row>
   </sheetData>
@@ -2900,16 +2886,16 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:S10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="21.08984375" style="1" customWidth="1"/>
-    <col min="2" max="19" width="11.54296875" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="1" width="21.109375" style="1" customWidth="1"/>
+    <col min="2" max="19" width="11.5546875" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.85">
       <c r="A1" s="55" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -2930,66 +2916,66 @@
       <c r="R1" s="56"/>
       <c r="S1" s="56"/>
     </row>
-    <row r="2" spans="1:19" ht="81" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:19" ht="79.2" x14ac:dyDescent="0.7">
       <c r="A2" s="145" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="118" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="119" t="s">
         <v>130</v>
       </c>
-      <c r="C2" s="119" t="s">
+      <c r="D2" s="118" t="s">
         <v>131</v>
       </c>
-      <c r="D2" s="118" t="s">
+      <c r="E2" s="92" t="s">
         <v>132</v>
       </c>
-      <c r="E2" s="92" t="s">
+      <c r="F2" s="93" t="s">
         <v>133</v>
       </c>
-      <c r="F2" s="93" t="s">
+      <c r="G2" s="92" t="s">
         <v>134</v>
       </c>
-      <c r="G2" s="92" t="s">
+      <c r="H2" s="92" t="s">
         <v>135</v>
       </c>
-      <c r="H2" s="92" t="s">
+      <c r="I2" s="93" t="s">
         <v>136</v>
       </c>
-      <c r="I2" s="93" t="s">
+      <c r="J2" s="92" t="s">
         <v>137</v>
       </c>
-      <c r="J2" s="92" t="s">
+      <c r="K2" s="92" t="s">
         <v>138</v>
       </c>
-      <c r="K2" s="92" t="s">
+      <c r="L2" s="93" t="s">
         <v>139</v>
       </c>
-      <c r="L2" s="93" t="s">
+      <c r="M2" s="92" t="s">
         <v>140</v>
       </c>
-      <c r="M2" s="92" t="s">
+      <c r="N2" s="92" t="s">
         <v>141</v>
       </c>
-      <c r="N2" s="92" t="s">
+      <c r="O2" s="93" t="s">
         <v>142</v>
       </c>
-      <c r="O2" s="93" t="s">
+      <c r="P2" s="92" t="s">
         <v>143</v>
       </c>
-      <c r="P2" s="92" t="s">
+      <c r="Q2" s="92" t="s">
         <v>144</v>
       </c>
-      <c r="Q2" s="92" t="s">
+      <c r="R2" s="93" t="s">
         <v>145</v>
       </c>
-      <c r="R2" s="93" t="s">
+      <c r="S2" s="92" t="s">
         <v>146</v>
       </c>
-      <c r="S2" s="92" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.9">
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A3" s="91" t="s">
         <v>34</v>
       </c>
@@ -3053,7 +3039,7 @@
         <v>1194</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A4" s="91" t="s">
         <v>33</v>
       </c>
@@ -3117,7 +3103,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A5" s="91" t="s">
         <v>32</v>
       </c>
@@ -3181,7 +3167,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A6" s="91" t="s">
         <v>31</v>
       </c>
@@ -3245,7 +3231,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A7" s="91" t="s">
         <v>30</v>
       </c>
@@ -3309,7 +3295,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="27.5" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="8" spans="1:19" ht="27" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A8" s="88" t="s">
         <v>4</v>
       </c>
@@ -3383,7 +3369,7 @@
         <v>2039</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A9" s="84" t="s">
         <v>28</v>
       </c>
@@ -3408,7 +3394,7 @@
       <c r="R9" s="81"/>
       <c r="S9" s="81"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.7">
       <c r="J10" s="80"/>
     </row>
   </sheetData>
@@ -3423,16 +3409,16 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="88.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="20.36328125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="1" width="88.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="20.33203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="55" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -3440,7 +3426,7 @@
       <c r="E1" s="55"/>
       <c r="F1" s="55"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.7">
       <c r="A2" s="62" t="s">
         <v>2</v>
       </c>
@@ -3460,7 +3446,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A3" s="97" t="s">
         <v>40</v>
       </c>
@@ -3480,9 +3466,9 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="36.65" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A4" s="60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B4" s="58">
         <v>1700</v>
@@ -3500,7 +3486,7 @@
         <v>2714</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A5" s="60" t="s">
         <v>39</v>
       </c>
@@ -3520,9 +3506,9 @@
         <v>45.946941783345601</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A6" s="96" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B6" s="96"/>
       <c r="C6" s="96"/>
@@ -3542,15 +3528,15 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="6" width="19.81640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.90625" style="1"/>
+    <col min="1" max="6" width="19.77734375" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24.65" customHeight="1" thickBot="1" x14ac:dyDescent="1">
+    <row r="1" spans="1:7" ht="24.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A1" s="55" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B1" s="56"/>
       <c r="C1" s="94"/>
@@ -3558,7 +3544,7 @@
       <c r="E1" s="94"/>
       <c r="F1" s="94"/>
     </row>
-    <row r="2" spans="1:7" ht="28.75" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A2" s="146"/>
       <c r="B2" s="105">
         <v>2020</v>
@@ -3576,7 +3562,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A3" s="147" t="s">
         <v>35</v>
       </c>
@@ -3596,7 +3582,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A4" s="104" t="s">
         <v>45</v>
       </c>
@@ -3616,7 +3602,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A5" s="104" t="s">
         <v>44</v>
       </c>
@@ -3636,7 +3622,7 @@
         <v>86.7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A6" s="104" t="s">
         <v>43</v>
       </c>
@@ -3656,7 +3642,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A7" s="104" t="s">
         <v>42</v>
       </c>
@@ -3676,7 +3662,7 @@
         <v>51.1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="27.5" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="8" spans="1:7" ht="27" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A8" s="103" t="s">
         <v>41</v>
       </c>
@@ -3696,7 +3682,7 @@
         <v>76.400000000000006</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A9" s="100" t="s">
         <v>28</v>
       </c>
@@ -3705,7 +3691,7 @@
       <c r="E9" s="98"/>
       <c r="F9" s="98"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.7">
       <c r="G10" s="95"/>
     </row>
   </sheetData>
@@ -3720,16 +3706,16 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
     <col min="1" max="1" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="11.36328125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.54296875" style="1"/>
+    <col min="2" max="6" width="11.33203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="50.4" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:6" ht="50.4" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="165" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B1" s="165"/>
       <c r="C1" s="165"/>
@@ -3737,7 +3723,7 @@
       <c r="E1" s="165"/>
       <c r="F1" s="165"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.7">
       <c r="A2" s="133" t="s">
         <v>50</v>
       </c>
@@ -3757,9 +3743,9 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.7">
       <c r="A3" s="104" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B3" s="58">
         <v>1700</v>
@@ -3777,7 +3763,7 @@
         <v>2390</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.7">
       <c r="A4" s="108" t="s">
         <v>49</v>
       </c>
@@ -3797,7 +3783,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="27.5" thickBot="1" x14ac:dyDescent="0.95">
+    <row r="5" spans="1:6" ht="27" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A5" s="107" t="s">
         <v>48</v>
       </c>
@@ -3817,7 +3803,7 @@
         <v>3.01255230125523</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.7">
       <c r="A6" s="106" t="s">
         <v>47</v>
       </c>
@@ -3839,24 +3825,24 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{620B2E2E-E71D-4040-86BE-8934D07E1F88}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
     <col min="1" max="1" width="31" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="13.54296875" style="1" customWidth="1"/>
-    <col min="5" max="6" width="11.54296875" style="1"/>
-    <col min="7" max="7" width="12.81640625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.54296875" style="1"/>
+    <col min="2" max="4" width="13.5546875" style="1" customWidth="1"/>
+    <col min="5" max="6" width="11.5546875" style="1"/>
+    <col min="7" max="7" width="12.77734375" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="166" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B1" s="166"/>
       <c r="C1" s="166"/>
       <c r="D1" s="166"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A2" s="62" t="s">
         <v>2</v>
       </c>
@@ -3870,7 +3856,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A3" s="60" t="s">
         <v>58</v>
       </c>
@@ -3884,7 +3870,7 @@
         <v>1939342</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A4" s="60" t="s">
         <v>57</v>
       </c>
@@ -3898,7 +3884,7 @@
         <v>4505</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A5" s="60" t="s">
         <v>56</v>
       </c>
@@ -3912,7 +3898,7 @@
         <v>1074208</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A6" s="60" t="s">
         <v>55</v>
       </c>
@@ -3926,7 +3912,7 @@
         <v>53787</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A7" s="60" t="s">
         <v>54</v>
       </c>
@@ -3940,7 +3926,7 @@
         <v>31608</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A8" s="60" t="s">
         <v>53</v>
       </c>
@@ -3954,7 +3940,7 @@
         <v>988822</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A9" s="125" t="s">
         <v>52</v>
       </c>
@@ -3968,7 +3954,7 @@
         <v>55.39</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A10" s="9" t="s">
         <v>51</v>
       </c>
@@ -3976,16 +3962,16 @@
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.7">
       <c r="D13" s="124"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.7">
       <c r="D14" s="124"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.7">
       <c r="D15" s="124"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.9">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.7">
       <c r="D17" s="124"/>
     </row>
   </sheetData>
@@ -4000,22 +3986,22 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{788F987F-F922-4486-BAC1-F0627BCE59A7}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="25.90625" style="1" customWidth="1"/>
-    <col min="2" max="4" width="14.81640625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="1" width="25.88671875" style="1" customWidth="1"/>
+    <col min="2" max="4" width="14.77734375" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="8"/>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
     </row>
-    <row r="2" spans="1:7" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.85">
       <c r="A2" s="33" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
@@ -4024,23 +4010,23 @@
       <c r="F2" s="128"/>
       <c r="G2" s="127"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A3" s="140" t="s">
         <v>59</v>
       </c>
       <c r="B3" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="D3" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="D3" s="29" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.9">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A4" s="97" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B4" s="58">
         <v>147</v>
@@ -4052,9 +4038,9 @@
         <v>157</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A5" s="97" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B5" s="58">
         <v>37</v>
@@ -4067,9 +4053,9 @@
       </c>
       <c r="F5" s="126"/>
     </row>
-    <row r="6" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A6" s="97" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B6" s="150">
         <v>25.170068027210899</v>
@@ -4081,7 +4067,7 @@
         <v>26.751592356687901</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A7" s="167" t="s">
         <v>51</v>
       </c>
@@ -4101,25 +4087,25 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC52C36-B447-461A-A3AB-32D330BCC6F5}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="24.90625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="24.88671875" style="1" customWidth="1"/>
     <col min="2" max="4" width="19" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.1796875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="11.54296875" style="1"/>
+    <col min="5" max="5" width="13.21875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="33" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A2" s="133" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" s="132">
         <v>2013</v>
@@ -4131,7 +4117,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A3" s="131" t="s">
         <v>58</v>
       </c>
@@ -4145,7 +4131,7 @@
         <v>1786448</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A4" s="131" t="s">
         <v>56</v>
       </c>
@@ -4159,9 +4145,9 @@
         <v>1272837</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A5" s="131" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5" s="130">
         <v>147</v>
@@ -4173,9 +4159,9 @@
         <v>176</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A6" s="131" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B6" s="130">
         <v>64</v>
@@ -4187,9 +4173,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A7" s="131" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="130">
         <v>438</v>
@@ -4201,9 +4187,9 @@
         <v>559</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A8" s="129" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8" s="151">
         <v>75.53</v>
@@ -4215,9 +4201,9 @@
         <v>0.71</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A9" s="167" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B9" s="167"/>
       <c r="C9" s="9"/>
@@ -4235,24 +4221,24 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF716CA6-EB93-4872-A88E-E3E7686AD6A1}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="31.90625" style="1" customWidth="1"/>
-    <col min="2" max="4" width="13.90625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="1" width="31.88671875" style="1" customWidth="1"/>
+    <col min="2" max="4" width="13.88671875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="33" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A2" s="62" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B2" s="29">
         <v>2013</v>
@@ -4264,7 +4250,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A3" s="135" t="s">
         <v>58</v>
       </c>
@@ -4278,7 +4264,7 @@
         <v>1786448</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A4" s="135" t="s">
         <v>56</v>
       </c>
@@ -4292,9 +4278,9 @@
         <v>1272837</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A5" s="135" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5" s="58">
         <v>147</v>
@@ -4306,9 +4292,9 @@
         <v>176</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A6" s="135" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B6" s="58">
         <v>64</v>
@@ -4320,9 +4306,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A7" s="135" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="58">
         <v>438</v>
@@ -4334,9 +4320,9 @@
         <v>559</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A8" s="134" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8" s="152">
         <v>0.75529999999999997</v>
@@ -4348,7 +4334,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A9" s="168" t="s">
         <v>51</v>
       </c>
@@ -4370,16 +4356,16 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="2" width="18.1796875" style="1" customWidth="1"/>
-    <col min="3" max="7" width="9.54296875" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="2" width="18.21875" style="1" customWidth="1"/>
+    <col min="3" max="7" width="9.5546875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="8"/>
@@ -4388,7 +4374,7 @@
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A2" s="12" t="s">
         <v>7</v>
       </c>
@@ -4411,7 +4397,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A3" s="14" t="s">
         <v>6</v>
       </c>
@@ -4434,7 +4420,7 @@
         <v>4312</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A4" s="14" t="s">
         <v>5</v>
       </c>
@@ -4457,7 +4443,7 @@
         <v>2786</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A5" s="12" t="s">
         <v>4</v>
       </c>
@@ -4480,7 +4466,7 @@
         <v>7098</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A6" s="10" t="s">
         <v>3</v>
       </c>
@@ -4500,23 +4486,23 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B05ABCB-A9D8-4F3C-A79A-E9A7F14450F7}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="31.453125" style="1" customWidth="1"/>
-    <col min="2" max="3" width="16.08984375" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="1" width="31.44140625" style="1" customWidth="1"/>
+    <col min="2" max="3" width="16.109375" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="82" customFormat="1" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:3" s="82" customFormat="1" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="137" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B1" s="138"/>
       <c r="C1" s="138"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A2" s="62" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B2" s="29">
         <v>2018</v>
@@ -4525,7 +4511,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A3" s="136" t="s">
         <v>58</v>
       </c>
@@ -4536,7 +4522,7 @@
         <v>1786448</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A4" s="97" t="s">
         <v>56</v>
       </c>
@@ -4547,7 +4533,7 @@
         <v>1272837</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A5" s="97" t="s">
         <v>53</v>
       </c>
@@ -4558,7 +4544,7 @@
         <v>1255463</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A6" s="97" t="s">
         <v>55</v>
       </c>
@@ -4569,9 +4555,9 @@
         <v>255615</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A7" s="97" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" s="152">
         <v>73</v>
@@ -4580,9 +4566,9 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A8" s="168" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B8" s="168"/>
       <c r="C8" s="9"/>
@@ -4601,16 +4587,16 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="2" width="21.1796875" style="1" customWidth="1"/>
-    <col min="3" max="7" width="11.6328125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="2" width="21.21875" style="1" customWidth="1"/>
+    <col min="3" max="7" width="11.6640625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="8"/>
@@ -4619,7 +4605,7 @@
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.7">
       <c r="A2" s="12" t="s">
         <v>10</v>
       </c>
@@ -4642,7 +4628,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.7">
       <c r="A3" s="18" t="s">
         <v>9</v>
       </c>
@@ -4665,7 +4651,7 @@
         <v>2034</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.7">
       <c r="A4" s="18" t="s">
         <v>8</v>
       </c>
@@ -4688,7 +4674,7 @@
         <v>5064</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.7">
       <c r="A5" s="17" t="s">
         <v>4</v>
       </c>
@@ -4711,7 +4697,7 @@
         <v>7098</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.7">
       <c r="A6" s="10" t="s">
         <v>3</v>
       </c>
@@ -4734,16 +4720,16 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="2" width="16.08984375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="16.109375" style="1" customWidth="1"/>
     <col min="3" max="7" width="14" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.54296875" style="1"/>
+    <col min="8" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="8"/>
@@ -4752,7 +4738,7 @@
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A2" s="12" t="s">
         <v>7</v>
       </c>
@@ -4775,7 +4761,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A3" s="14" t="s">
         <v>6</v>
       </c>
@@ -4798,7 +4784,7 @@
         <v>74534</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A4" s="14" t="s">
         <v>5</v>
       </c>
@@ -4821,7 +4807,7 @@
         <v>80611</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A5" s="12" t="s">
         <v>4</v>
       </c>
@@ -4844,7 +4830,7 @@
         <v>155145</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A6" s="10" t="s">
         <v>3</v>
       </c>
@@ -4866,15 +4852,15 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="2" width="21.36328125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="2" width="21.33203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="8"/>
@@ -4883,7 +4869,7 @@
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A2" s="12" t="s">
         <v>10</v>
       </c>
@@ -4906,7 +4892,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A3" s="14" t="s">
         <v>9</v>
       </c>
@@ -4929,7 +4915,7 @@
         <v>73602</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="22.25" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:7" ht="22.2" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A4" s="14" t="s">
         <v>8</v>
       </c>
@@ -4952,7 +4938,7 @@
         <v>81603</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A5" s="12" t="s">
         <v>4</v>
       </c>
@@ -4975,7 +4961,7 @@
         <v>155205</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.7">
       <c r="A6" s="10" t="s">
         <v>3</v>
       </c>
@@ -4994,14 +4980,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB79EA6F-52D8-4271-9F0B-1B8DE97AB912}">
   <dimension ref="A1:J5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="69.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="69.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -5013,7 +4999,7 @@
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
     </row>
-    <row r="2" spans="1:10" ht="27" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
         <v>2</v>
       </c>
@@ -5045,7 +5031,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="27" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
         <v>12</v>
       </c>
@@ -5077,9 +5063,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="27.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B4" s="32">
         <v>0.47</v>
@@ -5109,7 +5095,7 @@
         <v>0.81</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
         <v>11</v>
       </c>
@@ -5122,15 +5108,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CDBA7B6-7D99-4406-8139-02C0D51D2164}">
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.1796875" customWidth="1"/>
-    <col min="2" max="11" width="20.08984375" style="45" customWidth="1"/>
+    <col min="1" max="1" width="13.21875" customWidth="1"/>
+    <col min="2" max="11" width="20.109375" style="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="33" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -5143,42 +5129,42 @@
       <c r="J1" s="43"/>
       <c r="K1" s="43"/>
     </row>
-    <row r="2" spans="1:11" ht="108" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A2" s="139" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="D2" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="F2" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="G2" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="G2" s="34" t="s">
-        <v>72</v>
-      </c>
       <c r="H2" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="I2" s="34" t="s">
+      <c r="J2" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="34" t="s">
+      <c r="K2" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="K2" s="34" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="54" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A3" s="36" t="s">
         <v>14</v>
       </c>
@@ -5213,7 +5199,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="54" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:11" ht="52.8" x14ac:dyDescent="0.7">
       <c r="A4" s="39" t="s">
         <v>15</v>
       </c>
@@ -5248,7 +5234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="36" t="s">
         <v>16</v>
       </c>
@@ -5283,7 +5269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="36" t="s">
         <v>17</v>
       </c>
@@ -5318,7 +5304,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="36" t="s">
         <v>18</v>
       </c>
@@ -5353,7 +5339,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="36" t="s">
         <v>19</v>
       </c>
@@ -5388,7 +5374,7 @@
         <v>1.23</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="36" t="s">
         <v>20</v>
       </c>
@@ -5423,7 +5409,7 @@
         <v>1.39</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="81" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A10" s="36" t="s">
         <v>21</v>
       </c>
@@ -5458,7 +5444,7 @@
         <v>2.39</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="36" t="s">
         <v>22</v>
       </c>
@@ -5493,7 +5479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="54" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A12" s="36" t="s">
         <v>23</v>
       </c>
@@ -5528,7 +5514,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="54" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A13" s="36" t="s">
         <v>24</v>
       </c>
@@ -5563,7 +5549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="36" t="s">
         <v>25</v>
       </c>
@@ -5598,7 +5584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A15" s="36" t="s">
         <v>26</v>
       </c>
@@ -5631,7 +5617,7 @@
       </c>
       <c r="K15" s="37"/>
     </row>
-    <row r="16" spans="1:11" ht="27" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A16" s="35" t="s">
         <v>27</v>
       </c>
@@ -5666,7 +5652,7 @@
         <v>0.81</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="21" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:11" ht="21.6" x14ac:dyDescent="0.65">
       <c r="A17" s="10" t="s">
         <v>11</v>
       </c>
@@ -5692,31 +5678,31 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:S68"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="1" width="59.90625" style="1" customWidth="1"/>
-    <col min="2" max="4" width="11.36328125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="59.88671875" style="1" customWidth="1"/>
+    <col min="2" max="4" width="11.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="11.54296875" style="1"/>
+    <col min="20" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="29.5" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:19" ht="30" x14ac:dyDescent="0.85">
       <c r="A1" s="55" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -5737,66 +5723,66 @@
       <c r="R1" s="54"/>
       <c r="S1" s="54"/>
     </row>
-    <row r="2" spans="1:19" ht="54" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:19" ht="52.8" x14ac:dyDescent="0.7">
       <c r="A2" s="139" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="D2" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="F2" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="G2" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="G2" s="34" t="s">
+      <c r="H2" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="H2" s="34" t="s">
+      <c r="I2" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="I2" s="34" t="s">
+      <c r="J2" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="34" t="s">
+      <c r="K2" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="K2" s="34" t="s">
+      <c r="L2" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="L2" s="34" t="s">
+      <c r="M2" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="M2" s="34" t="s">
+      <c r="N2" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="N2" s="34" t="s">
+      <c r="O2" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="O2" s="34" t="s">
+      <c r="P2" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="P2" s="34" t="s">
+      <c r="Q2" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="Q2" s="34" t="s">
+      <c r="R2" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="R2" s="34" t="s">
+      <c r="S2" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="S2" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.9">
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A3" s="36" t="s">
         <v>14</v>
       </c>
@@ -5855,7 +5841,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A4" s="39" t="s">
         <v>15</v>
       </c>
@@ -5914,7 +5900,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A5" s="36" t="s">
         <v>16</v>
       </c>
@@ -5973,7 +5959,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A6" s="36" t="s">
         <v>17</v>
       </c>
@@ -6032,7 +6018,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A7" s="36" t="s">
         <v>18</v>
       </c>
@@ -6091,7 +6077,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A8" s="36" t="s">
         <v>19</v>
       </c>
@@ -6150,7 +6136,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A9" s="36" t="s">
         <v>20</v>
       </c>
@@ -6209,7 +6195,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="23.4" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="10" spans="1:19" ht="23.4" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A10" s="36" t="s">
         <v>21</v>
       </c>
@@ -6268,7 +6254,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A11" s="36" t="s">
         <v>22</v>
       </c>
@@ -6327,7 +6313,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A12" s="36" t="s">
         <v>23</v>
       </c>
@@ -6386,7 +6372,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A13" s="36" t="s">
         <v>24</v>
       </c>
@@ -6445,7 +6431,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A14" s="36" t="s">
         <v>25</v>
       </c>
@@ -6504,7 +6490,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A15" s="36" t="s">
         <v>26</v>
       </c>
@@ -6563,7 +6549,7 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A16" s="35" t="s">
         <v>27</v>
       </c>
@@ -6622,7 +6608,7 @@
         <v>2390</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="17" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A17" s="50" t="s">
         <v>28</v>
       </c>
@@ -6633,7 +6619,7 @@
       <c r="F17" s="9"/>
       <c r="H17" s="9"/>
     </row>
-    <row r="18" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="18" spans="1:8" ht="29.4" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A18" s="49"/>
       <c r="B18" s="49"/>
       <c r="C18" s="49"/>
@@ -6642,12 +6628,12 @@
       <c r="F18" s="9"/>
       <c r="H18" s="9"/>
     </row>
-    <row r="35" ht="18.75" customHeight="1" x14ac:dyDescent="0.9"/>
-    <row r="36" ht="37.75" customHeight="1" x14ac:dyDescent="0.9"/>
-    <row r="47" ht="18" customHeight="1" x14ac:dyDescent="0.9"/>
-    <row r="48" ht="19.399999999999999" customHeight="1" x14ac:dyDescent="0.9"/>
-    <row r="67" ht="18" customHeight="1" x14ac:dyDescent="0.9"/>
-    <row r="68" ht="18" customHeight="1" x14ac:dyDescent="0.9"/>
+    <row r="35" ht="18.75" customHeight="1" x14ac:dyDescent="0.7"/>
+    <row r="36" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.7"/>
+    <row r="47" ht="18" customHeight="1" x14ac:dyDescent="0.7"/>
+    <row r="48" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.7"/>
+    <row r="67" ht="18" customHeight="1" x14ac:dyDescent="0.7"/>
+    <row r="68" ht="18" customHeight="1" x14ac:dyDescent="0.7"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -6660,15 +6646,15 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:S8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="27" x14ac:dyDescent="0.9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="26.4" x14ac:dyDescent="0.7"/>
   <cols>
-    <col min="1" max="19" width="17.453125" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="11.54296875" style="1"/>
+    <col min="1" max="19" width="17.44140625" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="22.75" customHeight="1" x14ac:dyDescent="0.95">
+    <row r="1" spans="1:19" ht="22.8" customHeight="1" x14ac:dyDescent="0.85">
       <c r="A1" s="64" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B1" s="64"/>
       <c r="C1" s="64"/>
@@ -6689,66 +6675,66 @@
       <c r="R1" s="64"/>
       <c r="S1" s="64"/>
     </row>
-    <row r="2" spans="1:19" ht="54" x14ac:dyDescent="0.9">
+    <row r="2" spans="1:19" ht="52.8" x14ac:dyDescent="0.7">
       <c r="A2" s="140" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="110" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="111" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="111" t="s">
+      <c r="D2" s="110" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="I2" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="J2" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="K2" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="L2" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="M2" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="N2" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="110" t="s">
-        <v>84</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="G2" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="H2" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="I2" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="J2" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="K2" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="L2" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="M2" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="N2" s="34" t="s">
-        <v>102</v>
-      </c>
       <c r="O2" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="P2" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="P2" s="34" t="s">
+      <c r="Q2" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="Q2" s="34" t="s">
+      <c r="R2" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="R2" s="34" t="s">
+      <c r="S2" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="S2" s="34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.9">
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A3" s="60" t="s">
         <v>34</v>
       </c>
@@ -6806,7 +6792,7 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A4" s="60" t="s">
         <v>33</v>
       </c>
@@ -6864,7 +6850,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A5" s="60" t="s">
         <v>32</v>
       </c>
@@ -6924,7 +6910,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A6" s="60" t="s">
         <v>31</v>
       </c>
@@ -6982,7 +6968,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.9">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.7">
       <c r="A7" s="60" t="s">
         <v>30</v>
       </c>
@@ -7042,7 +7028,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="16.25" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="8" spans="1:19" ht="16.2" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A8" s="50" t="s">
         <v>28</v>
       </c>

</xml_diff>